<commit_message>
Updated da-DK and fr-FR
</commit_message>
<xml_diff>
--- a/assets/translations/French.France.fr-FR.xlsx
+++ b/assets/translations/French.France.fr-FR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11003"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mspitschan/Projects/LadenburgConsensusStatements/assets/translations/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lbickerstaff/Nextcloud/PhD/Documents/Other/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DBFEB50-8F61-7B49-95EA-230C20B4E55F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C5FDDBF-E82D-F34D-A17B-5B0153C21CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="920" yWindow="880" windowWidth="35080" windowHeight="22500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17280" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Contributors" sheetId="2" r:id="rId1"/>
@@ -377,9 +377,6 @@
     <t>L'exposition à la lumière peut être décrite par son intensité : la quantité totale d'énergie sur l'ensemble des longueurs d'onde de 380 à 780 nm, pondérée selon la fonction d'intérêt.</t>
   </si>
   <si>
-    <t>La lumière du jour a ce que l'on appelle un spectre large, avec beaucoup d'énergie sur nombreuses longueurs d'onde.</t>
-  </si>
-  <si>
     <t>Les différentes sources de lumière électrique (par exemple, les lampes LED ou fluorescentes, etc.) ont des spectres différents.</t>
   </si>
   <si>
@@ -665,9 +662,6 @@
     <t>Les différentes technologies des sources lumineuses utilisent divers matériaux pour convertir l’électricité en lumière. Selon les matériaux utilisés, l’intensité de la lumière se répartit de differentes manières sur l'ensemble des longueurs d’onde. Cette répartition de la lumière selon les longueurs d’onde est connue sous le nom de distribution spectrale.</t>
   </si>
   <si>
-    <t>Les ipRGCs expriment la mélanopsine (une protéine sensible à la lumière). Lorsque les ipRGCs sont exposés à une lumière vive, la mélanopsine est activée. Cette activation déclenche une voie neuronale qui bloque la production de mélatonine dans la glande pinéale.</t>
-  </si>
-  <si>
     <t>Principalement par le biais des ipRGCs, la lumière provoque la suppression de la mélatonine le soir et la nuit.</t>
   </si>
   <si>
@@ -678,6 +672,12 @@
   </si>
   <si>
     <t>0000-0002-6549-799X</t>
+  </si>
+  <si>
+    <t>La lumière du jour a ce que l'on appelle un spectre large, avec beaucoup d'énergie sur de nombreuses longueurs d'onde.</t>
+  </si>
+  <si>
+    <t>Les ipRGCs expriment la mélanopsine (une protéine sensible à la lumière). Lorsque les ipRGCs sont exposées à une lumière vive, la mélanopsine est activée. Cette activation déclenche une voie neuronale qui bloque la production de mélatonine dans la glande pinéale.</t>
   </si>
 </sst>
 </file>
@@ -1422,62 +1422,62 @@
     </row>
     <row r="2" spans="1:7" s="25" customFormat="1">
       <c r="A2" s="25" t="s">
+        <v>180</v>
+      </c>
+      <c r="B2" s="25" t="s">
         <v>181</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="C2" s="25" t="s">
         <v>182</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="D2" s="11" t="s">
         <v>183</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="E2" s="25" t="s">
         <v>184</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="F2" s="11" t="s">
         <v>185</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="25" customFormat="1">
       <c r="A3" s="25" t="s">
+        <v>186</v>
+      </c>
+      <c r="B3" s="25" t="s">
         <v>187</v>
       </c>
-      <c r="B3" s="25" t="s">
-        <v>188</v>
-      </c>
       <c r="C3" s="25" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D3" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>202</v>
+      </c>
+      <c r="F3" s="11" t="s">
         <v>203</v>
-      </c>
-      <c r="E3" s="25" t="s">
-        <v>204</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="4" spans="1:7" s="25" customFormat="1">
       <c r="A4" s="25" t="s">
+        <v>188</v>
+      </c>
+      <c r="B4" s="25" t="s">
         <v>189</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="C4" s="25" t="s">
         <v>190</v>
       </c>
-      <c r="C4" s="25" t="s">
+      <c r="D4" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="E4" s="25" t="s">
         <v>192</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="F4" s="25" t="s">
         <v>193</v>
-      </c>
-      <c r="F4" s="25" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="25" customFormat="1">
@@ -1556,13 +1556,13 @@
         <v>5</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="H2" s="8" t="s">
         <v>6</v>
       </c>
       <c r="I2" s="13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="85">
@@ -1583,13 +1583,13 @@
         <v>7</v>
       </c>
       <c r="G3" s="20" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H3" s="8" t="s">
         <v>8</v>
       </c>
       <c r="I3" s="14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="119">
@@ -1610,13 +1610,13 @@
         <v>9</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="H4" s="8" t="s">
         <v>10</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="136">
@@ -1631,19 +1631,19 @@
         <v>82</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>105</v>
+        <v>204</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>11</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H5" s="8" t="s">
         <v>83</v>
       </c>
       <c r="I5" s="13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="136">
@@ -1658,19 +1658,19 @@
         <v>67</v>
       </c>
       <c r="E6" s="21" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>12</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H6" s="8" t="s">
         <v>13</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="95">
@@ -1685,19 +1685,19 @@
         <v>14</v>
       </c>
       <c r="E7" s="16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>15</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="H7" s="8" t="s">
         <v>84</v>
       </c>
       <c r="I7" s="13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="102">
@@ -1705,7 +1705,7 @@
         <v>91</v>
       </c>
       <c r="B8" s="28" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C8" s="7">
         <v>7</v>
@@ -1714,19 +1714,19 @@
         <v>68</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>16</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H8" s="8" t="s">
         <v>75</v>
       </c>
       <c r="I8" s="13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="85">
@@ -1741,19 +1741,19 @@
         <v>78</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>79</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H9" s="8" t="s">
         <v>17</v>
       </c>
       <c r="I9" s="13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="57">
@@ -1768,19 +1768,19 @@
         <v>18</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>19</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>20</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="85">
@@ -1788,7 +1788,7 @@
         <v>92</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C11" s="7">
         <v>10</v>
@@ -1797,19 +1797,19 @@
         <v>21</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>22</v>
       </c>
       <c r="G11" s="12" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>23</v>
       </c>
       <c r="I11" s="13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="119">
@@ -1824,19 +1824,19 @@
         <v>24</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="F12" s="8" t="s">
         <v>25</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="H12" s="8" t="s">
         <v>26</v>
       </c>
       <c r="I12" s="13" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="76">
@@ -1851,19 +1851,19 @@
         <v>27</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>28</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H13" s="8" t="s">
         <v>29</v>
       </c>
       <c r="I13" s="13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="76">
@@ -1878,19 +1878,19 @@
         <v>85</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>30</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H14" s="8" t="s">
         <v>31</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="85">
@@ -1905,19 +1905,19 @@
         <v>32</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>33</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H15" s="8" t="s">
         <v>34</v>
       </c>
       <c r="I15" s="13" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="68">
@@ -1932,19 +1932,19 @@
         <v>35</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>86</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H16" s="8" t="s">
         <v>36</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="68">
@@ -1959,19 +1959,19 @@
         <v>37</v>
       </c>
       <c r="E17" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F17" s="8" t="s">
         <v>38</v>
       </c>
       <c r="G17" s="15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H17" s="8" t="s">
         <v>39</v>
       </c>
       <c r="I17" s="13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="68">
@@ -1986,19 +1986,19 @@
         <v>40</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F18" s="8" t="s">
         <v>41</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H18" s="8" t="s">
         <v>87</v>
       </c>
       <c r="I18" s="13" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="68">
@@ -2013,19 +2013,19 @@
         <v>42</v>
       </c>
       <c r="E19" s="16" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F19" s="8" t="s">
         <v>43</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H19" s="8" t="s">
         <v>44</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="68">
@@ -2040,19 +2040,19 @@
         <v>45</v>
       </c>
       <c r="E20" s="15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>46</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H20" s="8" t="s">
         <v>47</v>
       </c>
       <c r="I20" s="13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="95">
@@ -2067,19 +2067,19 @@
         <v>80</v>
       </c>
       <c r="E21" s="16" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F21" s="8" t="s">
         <v>48</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H21" s="8" t="s">
         <v>49</v>
       </c>
       <c r="I21" s="13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="68">
@@ -2087,7 +2087,7 @@
         <v>93</v>
       </c>
       <c r="B22" s="28" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C22" s="7">
         <v>21</v>
@@ -2096,19 +2096,19 @@
         <v>88</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>50</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H22" s="8" t="s">
         <v>51</v>
       </c>
       <c r="I22" s="13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="76">
@@ -2123,19 +2123,19 @@
         <v>52</v>
       </c>
       <c r="E23" s="16" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F23" s="8" t="s">
         <v>53</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H23" s="8" t="s">
         <v>54</v>
       </c>
       <c r="I23" s="13" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="68">
@@ -2150,19 +2150,19 @@
         <v>55</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F24" s="8" t="s">
         <v>56</v>
       </c>
       <c r="G24" s="16" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H24" s="8" t="s">
         <v>57</v>
       </c>
       <c r="I24" s="13" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="57">
@@ -2170,7 +2170,7 @@
         <v>94</v>
       </c>
       <c r="B25" s="28" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C25" s="7">
         <v>24</v>
@@ -2179,19 +2179,19 @@
         <v>58</v>
       </c>
       <c r="E25" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F25" s="8" t="s">
         <v>59</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H25" s="8" t="s">
         <v>60</v>
       </c>
       <c r="I25" s="13" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="119">
@@ -2206,19 +2206,19 @@
         <v>61</v>
       </c>
       <c r="E26" s="16" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F26" s="8" t="s">
         <v>62</v>
       </c>
       <c r="G26" s="16" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H26" s="8" t="s">
         <v>63</v>
       </c>
       <c r="I26" s="13" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="120" thickBot="1">
@@ -2233,19 +2233,19 @@
         <v>64</v>
       </c>
       <c r="E27" s="23" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>65</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H27" s="10" t="s">
         <v>66</v>
       </c>
       <c r="I27" s="24" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -2276,7 +2276,7 @@
         <v>96</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="68">
@@ -2284,7 +2284,7 @@
         <v>97</v>
       </c>
       <c r="B3" s="28" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="85">
@@ -2292,7 +2292,7 @@
         <v>98</v>
       </c>
       <c r="B4" s="28" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="85">
@@ -2300,7 +2300,7 @@
         <v>99</v>
       </c>
       <c r="B5" s="28" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="102">
@@ -2308,7 +2308,7 @@
         <v>100</v>
       </c>
       <c r="B6" s="28" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>

</xml_diff>